<commit_message>
docs: remove test case statistics sheet
</commit_message>
<xml_diff>
--- a/docs/电商订单管理系统测试用例.xlsx
+++ b/docs/电商订单管理系统测试用例.xlsx
@@ -2,8 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="1" r:id="R8d9b7984638d4102"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="用例统计" sheetId="2" r:id="R49f1d724a8054b36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能测试用例" sheetId="1" r:id="R9abd2eec379143f4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2604,98 +2603,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">已发货订单界面没有发货入口，订单仍为已发货</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">电商订单管理系统 · 测试用例统计</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">统计结果会随“功能测试用例”中的优先级、模块和执行状态自动更新；缺陷闭环按当前回归记录汇总</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">用例总数</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P0用例</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">未执行</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已通过</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">失败</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">通过率</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">用例数</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">占比</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">数量/比例</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">说明</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已执行且符合预期</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">需关联缺陷并复测</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">尚未执行</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">阻塞</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">因环境或依赖无法执行</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已执行</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">通过＋失败＋阻塞</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">执行率</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已执行/用例总数</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">缺陷闭环</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">数量</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">累计发现</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">按回归记录中的首次失败统计</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已关闭</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已修复并完成回归测试</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">执行与回归填写说明</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">1. “执行状态”记录最终结论；失败修复并复测后改为“通过”。
-2. 原失败现象、缺陷编号、回归日期和关闭结论统一写入“回归记录”，不要删除失败历史。
-3. “实际结果”只填写本次真实表现；并发用例应同时保留 JMeter 结果截图或报告。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">来源：最新测试执行记录与原《电商订单管理系统.xmind》测试点分析（更新于2026-07-21）</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -7931,484 +7838,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad9e739c09b24a0c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd933333a2374649"/>
   </x:tableParts>
 </x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
-  <x:cols>
-    <x:col min="1" max="1" width="17" customWidth="1"/>
-    <x:col min="2" max="3" width="12" customWidth="1"/>
-    <x:col min="4" max="4" width="4" customWidth="1"/>
-    <x:col min="5" max="5" width="17" customWidth="1"/>
-    <x:col min="6" max="6" width="14" customWidth="1"/>
-    <x:col min="7" max="7" width="30" customWidth="1"/>
-    <x:col min="8" max="8" width="15" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="1" t="s">
-        <x:v>791</x:v>
-      </x:c>
-      <x:c r="B1" s="1"/>
-      <x:c r="C1" s="1"/>
-      <x:c r="D1" s="1"/>
-      <x:c r="E1" s="1"/>
-      <x:c r="F1" s="1"/>
-      <x:c r="G1" s="1"/>
-      <x:c r="H1" s="1"/>
-    </x:row>
-    <x:row r="2" ht="14.5">
-      <x:c r="A2" s="2" t="s">
-        <x:v>792</x:v>
-      </x:c>
-      <x:c r="B2" s="2"/>
-      <x:c r="C2" s="2"/>
-      <x:c r="D2" s="2"/>
-      <x:c r="E2" s="2"/>
-      <x:c r="F2" s="2"/>
-      <x:c r="G2" s="2"/>
-      <x:c r="H2" s="2"/>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="3" t="s">
-        <x:v>793</x:v>
-      </x:c>
-      <x:c r="B3" s="4" t="n">
-        <x:f>COUNTA('功能测试用例'!$A$2:$A$117)</x:f>
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="C3" s="5"/>
-      <x:c r="D3" s="3" t="s">
-        <x:v>794</x:v>
-      </x:c>
-      <x:c r="E3" s="4" t="n">
-        <x:f>COUNTIF('功能测试用例'!$E$2:$E$117,"P0")</x:f>
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F3" s="5"/>
-      <x:c r="G3" s="3" t="s">
-        <x:v>795</x:v>
-      </x:c>
-      <x:c r="H3" s="4" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"未执行")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="28" customHeight="1">
-      <x:c r="A4" s="5"/>
-      <x:c r="B4" s="5"/>
-      <x:c r="C4" s="5"/>
-      <x:c r="D4" s="5"/>
-      <x:c r="E4" s="5"/>
-      <x:c r="F4" s="5"/>
-      <x:c r="G4" s="5"/>
-      <x:c r="H4" s="5"/>
-    </x:row>
-    <x:row r="5" ht="28" customHeight="1">
-      <x:c r="A5" s="3" t="s">
-        <x:v>796</x:v>
-      </x:c>
-      <x:c r="B5" s="4" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"通过")</x:f>
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="C5" s="5"/>
-      <x:c r="D5" s="3" t="s">
-        <x:v>797</x:v>
-      </x:c>
-      <x:c r="E5" s="4" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"失败")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F5" s="5"/>
-      <x:c r="G5" s="3" t="s">
-        <x:v>798</x:v>
-      </x:c>
-      <x:c r="H5" s="6" t="n">
-        <x:f>IF(B3=0,0,B5/B3)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="14.5">
-      <x:c r="A6" s="7"/>
-      <x:c r="B6" s="7"/>
-      <x:c r="C6" s="7"/>
-      <x:c r="D6" s="7"/>
-      <x:c r="E6" s="7"/>
-      <x:c r="F6" s="7"/>
-      <x:c r="G6" s="7"/>
-      <x:c r="H6" s="7"/>
-    </x:row>
-    <x:row r="7" ht="14.5">
-      <x:c r="A7" s="7"/>
-      <x:c r="B7" s="7"/>
-      <x:c r="C7" s="7"/>
-      <x:c r="D7" s="7"/>
-      <x:c r="E7" s="7"/>
-      <x:c r="F7" s="7"/>
-      <x:c r="G7" s="7"/>
-      <x:c r="H7" s="7"/>
-    </x:row>
-    <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="8" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B8" s="8" t="s">
-        <x:v>799</x:v>
-      </x:c>
-      <x:c r="C8" s="8" t="s">
-        <x:v>800</x:v>
-      </x:c>
-      <x:c r="D8" s="7"/>
-      <x:c r="E8" s="9" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="F8" s="9" t="s">
-        <x:v>801</x:v>
-      </x:c>
-      <x:c r="G8" s="9" t="s">
-        <x:v>802</x:v>
-      </x:c>
-      <x:c r="H8" s="7"/>
-    </x:row>
-    <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="10" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B9" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A9)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C9" s="11" t="n">
-        <x:f t="shared" ref="C9:C18" si="0">IF($B$3=0,0,B9/$B$3)</x:f>
-        <x:v>0.1206896551724138</x:v>
-      </x:c>
-      <x:c r="D9" s="7"/>
-      <x:c r="E9" s="12" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F9" s="12" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"通过")</x:f>
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="G9" s="13" t="s">
-        <x:v>803</x:v>
-      </x:c>
-      <x:c r="H9" s="7"/>
-    </x:row>
-    <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="10" t="s">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="B10" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A10)</x:f>
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C10" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.0689655172413793</x:v>
-      </x:c>
-      <x:c r="D10" s="7"/>
-      <x:c r="E10" s="12" t="s">
-        <x:v>797</x:v>
-      </x:c>
-      <x:c r="F10" s="12" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"失败")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G10" s="13" t="s">
-        <x:v>804</x:v>
-      </x:c>
-      <x:c r="H10" s="7"/>
-    </x:row>
-    <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="10" t="s">
-        <x:v>159</x:v>
-      </x:c>
-      <x:c r="B11" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A11)</x:f>
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="C11" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.0948275862068965</x:v>
-      </x:c>
-      <x:c r="D11" s="7"/>
-      <x:c r="E11" s="12" t="s">
-        <x:v>795</x:v>
-      </x:c>
-      <x:c r="F11" s="12" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"未执行")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G11" s="13" t="s">
-        <x:v>805</x:v>
-      </x:c>
-      <x:c r="H11" s="7"/>
-    </x:row>
-    <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="10" t="s">
-        <x:v>238</x:v>
-      </x:c>
-      <x:c r="B12" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A12)</x:f>
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="C12" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.112068965517241</x:v>
-      </x:c>
-      <x:c r="D12" s="7"/>
-      <x:c r="E12" s="12" t="s">
-        <x:v>806</x:v>
-      </x:c>
-      <x:c r="F12" s="12" t="n">
-        <x:f>COUNTIF('功能测试用例'!$J$2:$J$117,"阻塞")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G12" s="13" t="s">
-        <x:v>807</x:v>
-      </x:c>
-      <x:c r="H12" s="7"/>
-    </x:row>
-    <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="10" t="s">
-        <x:v>328</x:v>
-      </x:c>
-      <x:c r="B13" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A13)</x:f>
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C13" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.0775862068965517</x:v>
-      </x:c>
-      <x:c r="D13" s="7"/>
-      <x:c r="E13" s="12" t="s">
-        <x:v>808</x:v>
-      </x:c>
-      <x:c r="F13" s="12" t="n">
-        <x:f>F9+F10+F12</x:f>
-        <x:v>116</x:v>
-      </x:c>
-      <x:c r="G13" s="13" t="s">
-        <x:v>809</x:v>
-      </x:c>
-      <x:c r="H13" s="7"/>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="10" t="s">
-        <x:v>388</x:v>
-      </x:c>
-      <x:c r="B14" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A14)</x:f>
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="C14" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.181034482758621</x:v>
-      </x:c>
-      <x:c r="D14" s="7"/>
-      <x:c r="E14" s="12" t="s">
-        <x:v>810</x:v>
-      </x:c>
-      <x:c r="F14" s="14" t="n">
-        <x:f>IF($B$3=0,0,F13/$B$3)</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G14" s="13" t="s">
-        <x:v>811</x:v>
-      </x:c>
-      <x:c r="H14" s="7"/>
-    </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="10" t="s">
-        <x:v>532</x:v>
-      </x:c>
-      <x:c r="B15" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A15)</x:f>
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C15" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.0172413793103448</x:v>
-      </x:c>
-      <x:c r="D15" s="7"/>
-      <x:c r="E15" s="15"/>
-      <x:c r="F15" s="15"/>
-      <x:c r="G15" s="15"/>
-      <x:c r="H15" s="7"/>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="10" t="s">
-        <x:v>547</x:v>
-      </x:c>
-      <x:c r="B16" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A16)</x:f>
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="C16" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.146551724137931</x:v>
-      </x:c>
-      <x:c r="D16" s="7"/>
-      <x:c r="E16" s="16" t="s">
-        <x:v>812</x:v>
-      </x:c>
-      <x:c r="F16" s="16" t="s">
-        <x:v>813</x:v>
-      </x:c>
-      <x:c r="G16" s="16" t="s">
-        <x:v>802</x:v>
-      </x:c>
-      <x:c r="H16" s="7"/>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="10" t="s">
-        <x:v>658</x:v>
-      </x:c>
-      <x:c r="B17" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A17)</x:f>
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="C17" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.0603448275862069</x:v>
-      </x:c>
-      <x:c r="D17" s="7"/>
-      <x:c r="E17" s="17" t="s">
-        <x:v>814</x:v>
-      </x:c>
-      <x:c r="F17" s="17">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G17" s="18" t="s">
-        <x:v>815</x:v>
-      </x:c>
-      <x:c r="H17" s="7"/>
-    </x:row>
-    <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="10" t="s">
-        <x:v>704</x:v>
-      </x:c>
-      <x:c r="B18" s="10" t="n">
-        <x:f>COUNTIF('功能测试用例'!$B$2:$B$117,A18)</x:f>
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="C18" s="11">
-        <x:f t="shared" si="0"/>
-        <x:v>0.120689655172414</x:v>
-      </x:c>
-      <x:c r="D18" s="7"/>
-      <x:c r="E18" s="17" t="s">
-        <x:v>816</x:v>
-      </x:c>
-      <x:c r="F18" s="17">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G18" s="18" t="s">
-        <x:v>817</x:v>
-      </x:c>
-      <x:c r="H18" s="7"/>
-    </x:row>
-    <x:row r="19" ht="14.5">
-      <x:c r="A19" s="7"/>
-      <x:c r="B19" s="7"/>
-      <x:c r="C19" s="7"/>
-      <x:c r="D19" s="7"/>
-      <x:c r="E19" s="7"/>
-      <x:c r="F19" s="7"/>
-      <x:c r="G19" s="7"/>
-      <x:c r="H19" s="7"/>
-    </x:row>
-    <x:row r="20" ht="14.5">
-      <x:c r="A20" s="7"/>
-      <x:c r="B20" s="7"/>
-      <x:c r="C20" s="7"/>
-      <x:c r="D20" s="7"/>
-      <x:c r="E20" s="7"/>
-      <x:c r="F20" s="7"/>
-      <x:c r="G20" s="7"/>
-      <x:c r="H20" s="7"/>
-    </x:row>
-    <x:row r="21" ht="16.5">
-      <x:c r="A21" s="19" t="s">
-        <x:v>818</x:v>
-      </x:c>
-      <x:c r="B21" s="19"/>
-      <x:c r="C21" s="19"/>
-      <x:c r="D21" s="19"/>
-      <x:c r="E21" s="19"/>
-      <x:c r="F21" s="19"/>
-      <x:c r="G21" s="19"/>
-      <x:c r="H21" s="19"/>
-    </x:row>
-    <x:row r="22" ht="28" customHeight="1">
-      <x:c r="A22" s="20" t="s">
-        <x:v>819</x:v>
-      </x:c>
-      <x:c r="B22" s="20"/>
-      <x:c r="C22" s="20"/>
-      <x:c r="D22" s="20"/>
-      <x:c r="E22" s="20"/>
-      <x:c r="F22" s="20"/>
-      <x:c r="G22" s="20"/>
-      <x:c r="H22" s="20"/>
-    </x:row>
-    <x:row r="23" ht="28" customHeight="1">
-      <x:c r="A23" s="20"/>
-      <x:c r="B23" s="20"/>
-      <x:c r="C23" s="20"/>
-      <x:c r="D23" s="20"/>
-      <x:c r="E23" s="20"/>
-      <x:c r="F23" s="20"/>
-      <x:c r="G23" s="20"/>
-      <x:c r="H23" s="20"/>
-    </x:row>
-    <x:row r="24" ht="28" customHeight="1">
-      <x:c r="A24" s="20"/>
-      <x:c r="B24" s="20"/>
-      <x:c r="C24" s="20"/>
-      <x:c r="D24" s="20"/>
-      <x:c r="E24" s="20"/>
-      <x:c r="F24" s="20"/>
-      <x:c r="G24" s="20"/>
-      <x:c r="H24" s="20"/>
-    </x:row>
-    <x:row r="25" ht="14.5">
-      <x:c r="A25" s="7"/>
-      <x:c r="B25" s="7"/>
-      <x:c r="C25" s="7"/>
-      <x:c r="D25" s="7"/>
-      <x:c r="E25" s="7"/>
-      <x:c r="F25" s="7"/>
-      <x:c r="G25" s="7"/>
-      <x:c r="H25" s="7"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="21" t="s">
-        <x:v>820</x:v>
-      </x:c>
-      <x:c r="B26" s="21"/>
-      <x:c r="C26" s="21"/>
-      <x:c r="D26" s="21"/>
-      <x:c r="E26" s="21"/>
-      <x:c r="F26" s="21"/>
-      <x:c r="G26" s="21"/>
-      <x:c r="H26" s="21"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
-    <x:mergeCell ref="A2:H2"/>
-    <x:mergeCell ref="A21:H21"/>
-    <x:mergeCell ref="A26:H26"/>
-    <x:mergeCell ref="A22:H24"/>
-  </x:mergeCells>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</x:worksheet>
 </file>
</xml_diff>